<commit_message>
Refactor automation theo POM và cập nhật report
</commit_message>
<xml_diff>
--- a/documents/Automation_Manual_Comparison.xlsx
+++ b/documents/Automation_Manual_Comparison.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong quan" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bao phu chuc nang" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doi chieu chi tiet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sau refactor POM" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -42,11 +43,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,18 +72,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -164,6 +154,63 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ComparisonOverview" displayName="ComparisonOverview" ref="A1:B10" headerRowCount="1">
+  <autoFilter ref="A1:B10"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="Chỉ số"/>
+    <tableColumn id="2" name="Giá trị"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CoverageByFunction" displayName="CoverageByFunction" ref="A1:E13" headerRowCount="1">
+  <autoFilter ref="A1:E13"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Chức năng"/>
+    <tableColumn id="2" name="Manual test cases"/>
+    <tableColumn id="3" name="Automation scripts"/>
+    <tableColumn id="4" name="Runtime pass"/>
+    <tableColumn id="5" name="Chưa chạy"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ComparisonDetail" displayName="ComparisonDetail" ref="A1:K33" headerRowCount="1">
+  <autoFilter ref="A1:K33"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="Mã test case"/>
+    <tableColumn id="2" name="Chức năng"/>
+    <tableColumn id="3" name="Độ ưu tiên"/>
+    <tableColumn id="4" name="Manual result"/>
+    <tableColumn id="5" name="Automation script"/>
+    <tableColumn id="6" name="Dry-run sau POM"/>
+    <tableColumn id="7" name="Runtime result"/>
+    <tableColumn id="8" name="Môi trường chạy"/>
+    <tableColumn id="9" name="Nhận xét"/>
+    <tableColumn id="10" name="File test"/>
+    <tableColumn id="11" name="Resource chính"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="PomComparison" displayName="PomComparison" ref="A1:C6" headerRowCount="1">
+  <autoFilter ref="A1:C6"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Nhóm"/>
+    <tableColumn id="2" name="Trước refactor"/>
+    <tableColumn id="3" name="Sau refactor POM"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -455,41 +502,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Chi so</t>
+          <t>Chỉ số</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Gia tri</t>
+          <t>Giá trị</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ngon ngu su dung</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Tieng Viet khong dau de tranh loi encoding; chi giu ma test case va duong dan file la dinh danh ky thuat.</t>
-        </is>
+          <t>Tổng số manual test cases</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Tong so test case kiem thu thu cong</t>
+          <t>Manual Pass</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -499,7 +544,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>So test case thu cong dat</t>
+          <t>Automation scripts</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -509,7 +554,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>So test case da co kiem thu tu dong</t>
+          <t>Runtime Pass</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -519,7 +564,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>So test case dat buoc kiem tra cu phap</t>
+          <t>Dry-run sau POM Pass</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -529,17 +574,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>So test case chay that dat</t>
+          <t>Fail</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>So test case chua chay that</t>
+          <t>Test cases chưa automation</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -549,37 +594,32 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Ty le bao phu bang kiem thu tu dong</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>1</v>
+          <t>Tỷ lệ bao phủ automation</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Ty le da xac nhan bang chay that</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Ghi chu moi truong</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>24 test case chay production theo nhom nho; 8 test case lien quan diem danh, thoi khoa bieu va bao cao chay local tai http://localhost:8080.</t>
+          <t>Tỷ lệ khớp manual/automation</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -593,43 +633,43 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Chuc nang</t>
+          <t>Chức năng</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>So test case thu cong</t>
+          <t>Manual test cases</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Automation scripts</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Chay that dat</t>
+          <t>Runtime pass</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Chua chay that</t>
+          <t>Chưa chạy</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Bao cao</t>
+          <t>Báo cáo</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
@@ -648,7 +688,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Dang ky</t>
+          <t>Đăng ký</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
@@ -667,7 +707,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Dang nhap</t>
+          <t>Đăng nhập</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -686,7 +726,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Dang xuat</t>
+          <t>Đăng xuất</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
@@ -705,7 +745,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Diem danh</t>
+          <t>Điểm danh</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -724,7 +764,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Khoa diem danh</t>
+          <t>Khóa điểm danh</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -743,7 +783,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lop hoc</t>
+          <t>Lớp học</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
@@ -762,7 +802,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Nhap danh sach sinh vien</t>
+          <t>Nhập danh sách sinh viên</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -781,7 +821,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Phan cong tiet hoc</t>
+          <t>Phân công tiết học</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
@@ -800,7 +840,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Phan quyen</t>
+          <t>Phân quyền</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
@@ -819,7 +859,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Sinh vien</t>
+          <t>Sinh viên</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
@@ -838,7 +878,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Thoi khoa bieu</t>
+          <t>Thời khóa biểu</t>
         </is>
       </c>
       <c r="B13" s="2" t="n">
@@ -856,6 +896,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -865,70 +908,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="51" customWidth="1" min="8" max="8"/>
-    <col width="56" customWidth="1" min="9" max="9"/>
-    <col width="62" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Ma test case</t>
+          <t>Mã test case</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Chuc nang</t>
+          <t>Chức năng</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Do uu tien</t>
+          <t>Độ ưu tiên</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Ket qua thu cong</t>
+          <t>Manual result</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Trang thai kiem thu tu dong</t>
+          <t>Automation script</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Kiem tra cu phap</t>
+          <t>Dry-run sau POM</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Chay that</t>
+          <t>Runtime result</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Moi truong chay</t>
+          <t>Môi trường chạy</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Nhan xet so sanh</t>
+          <t>Nhận xét</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>File kiem thu tu dong</t>
+          <t>File test</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Resource chính</t>
         </is>
       </c>
     </row>
@@ -940,7 +989,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Dang nhap</t>
+          <t>Đăng nhập</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -950,22 +999,22 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -975,12 +1024,17 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/login_smoke.robot</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/login_page.resource</t>
         </is>
       </c>
     </row>
@@ -992,7 +1046,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Dang nhap</t>
+          <t>Đăng nhập</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1002,22 +1056,22 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1027,12 +1081,17 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/login_smoke.robot</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/login_page.resource</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1103,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Dang nhap</t>
+          <t>Đăng nhập</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1054,22 +1113,22 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1079,12 +1138,17 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/login_smoke.robot</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/login_page.resource</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1160,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Dang nhap</t>
+          <t>Đăng nhập</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1106,22 +1170,22 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1131,12 +1195,17 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/login_smoke.robot</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/login_page.resource</t>
         </is>
       </c>
     </row>
@@ -1148,32 +1217,32 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Dang nhap</t>
+          <t>Đăng nhập</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1183,12 +1252,17 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/login_smoke.robot</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/login_page.resource</t>
         </is>
       </c>
     </row>
@@ -1200,32 +1274,32 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Dang xuat</t>
+          <t>Đăng xuất</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1235,12 +1309,17 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/login_smoke.robot</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/dashboard_page.resource</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1331,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Phan quyen</t>
+          <t>Phân quyền</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1262,22 +1341,22 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1287,12 +1366,17 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/role_regression.robot</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/dashboard_page.resource</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1388,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Phan quyen</t>
+          <t>Phân quyền</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1314,22 +1398,22 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1339,12 +1423,17 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/role_regression.robot</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/dashboard_page.resource</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1445,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Phan quyen</t>
+          <t>Phân quyền</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1366,22 +1455,22 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1391,12 +1480,17 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/role_regression.robot</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/dashboard_page.resource</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1502,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Lop hoc</t>
+          <t>Lớp học</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1418,22 +1512,22 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1443,12 +1537,17 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/class_student_import_regression.robot</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/class_page.resource</t>
         </is>
       </c>
     </row>
@@ -1460,32 +1559,32 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Lop hoc</t>
+          <t>Lớp học</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1495,12 +1594,17 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/class_student_import_regression.robot</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/class_page.resource</t>
         </is>
       </c>
     </row>
@@ -1512,32 +1616,32 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Lop hoc</t>
+          <t>Lớp học</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1547,12 +1651,17 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/class_student_import_regression.robot</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/class_page.resource</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1673,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Sinh vien</t>
+          <t>Sinh viên</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1574,22 +1683,22 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1599,12 +1708,17 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/class_student_import_regression.robot</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/student_page.resource</t>
         </is>
       </c>
     </row>
@@ -1616,32 +1730,32 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Sinh vien</t>
+          <t>Sinh viên</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1651,12 +1765,17 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/services/api_flows.resource</t>
         </is>
       </c>
     </row>
@@ -1668,32 +1787,32 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Sinh vien</t>
+          <t>Sinh viên</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1703,12 +1822,17 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/services/api_flows.resource</t>
         </is>
       </c>
     </row>
@@ -1720,32 +1844,32 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Nhap danh sach sinh vien</t>
+          <t>Nhập danh sách sinh viên</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1755,12 +1879,17 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/services/api_flows.resource</t>
         </is>
       </c>
     </row>
@@ -1772,32 +1901,32 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Nhap danh sach sinh vien</t>
+          <t>Nhập danh sách sinh viên</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1807,12 +1936,17 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/class_student_import_regression.robot</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/student_page.resource</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1958,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Diem danh</t>
+          <t>Điểm danh</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1834,22 +1968,22 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1859,12 +1993,17 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/attendance_schedule_report_regression.robot</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/attendance_page.resource</t>
         </is>
       </c>
     </row>
@@ -1876,32 +2015,32 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Diem danh</t>
+          <t>Điểm danh</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1911,12 +2050,17 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/attendance_schedule_report_regression.robot</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/attendance_page.resource</t>
         </is>
       </c>
     </row>
@@ -1928,7 +2072,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Khoa diem danh</t>
+          <t>Khóa điểm danh</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1938,22 +2082,22 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1963,12 +2107,17 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/attendance_schedule_report_regression.robot</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/attendance_page.resource</t>
         </is>
       </c>
     </row>
@@ -1980,32 +2129,32 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Dang ky</t>
+          <t>Đăng ký</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2015,12 +2164,17 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/register_page.resource</t>
         </is>
       </c>
     </row>
@@ -2032,32 +2186,32 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Dang ky</t>
+          <t>Đăng ký</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2067,12 +2221,17 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/register_page.resource</t>
         </is>
       </c>
     </row>
@@ -2084,32 +2243,32 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Dang ky</t>
+          <t>Đăng ký</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2119,12 +2278,17 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/register_page.resource</t>
         </is>
       </c>
     </row>
@@ -2136,32 +2300,32 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Dang ky</t>
+          <t>Đăng ký</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2171,12 +2335,17 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/register_page.resource</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2357,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Phan cong tiet hoc</t>
+          <t>Phân công tiết học</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2198,22 +2367,22 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -2223,12 +2392,17 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/attendance_schedule_report_regression.robot</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/schedule_page.resource</t>
         </is>
       </c>
     </row>
@@ -2240,32 +2414,32 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Phan cong tiet hoc</t>
+          <t>Phân công tiết học</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2275,12 +2449,17 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/services/api_flows.resource</t>
         </is>
       </c>
     </row>
@@ -2292,32 +2471,32 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Phan cong tiet hoc</t>
+          <t>Phân công tiết học</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2327,12 +2506,17 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/services/api_flows.resource</t>
         </is>
       </c>
     </row>
@@ -2344,32 +2528,32 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Thoi khoa bieu</t>
+          <t>Thời khóa biểu</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2379,12 +2563,17 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/attendance_schedule_report_regression.robot</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/timetable_page.resource</t>
         </is>
       </c>
     </row>
@@ -2396,32 +2585,32 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Thoi khoa bieu</t>
+          <t>Thời khóa biểu</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2431,12 +2620,17 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/attendance_schedule_report_regression.robot</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/timetable_page.resource</t>
         </is>
       </c>
     </row>
@@ -2448,32 +2642,32 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Bao cao</t>
+          <t>Báo cáo</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2483,12 +2677,17 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/attendance_schedule_report_regression.robot</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/report_page.resource</t>
         </is>
       </c>
     </row>
@@ -2500,32 +2699,32 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Bao cao</t>
+          <t>Báo cáo</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2535,12 +2734,17 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/attendance_schedule_report_regression.robot</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/pages/report_page.resource</t>
         </is>
       </c>
     </row>
@@ -2552,32 +2756,32 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Bao cao</t>
+          <t>Báo cáo</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Trung binh</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Da co kiem thu tu dong</t>
+          <t>Đã có</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Dat</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>Dat</t>
+          <t>Đạt</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Đạt</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -2587,16 +2791,148 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>Ket qua thu cong dat va kiem thu tu dong chay that dat</t>
+          <t>Manual và automation đều Pass trong phạm vi test hiện tại</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
           <t>Automation/tests/remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Automation/resources/services/api_flows.resource</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nhóm</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Trước refactor</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Sau refactor POM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Test suite</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Có đủ 5 suite automation</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Giữ nguyên 5 suite automation</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Locator</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Một phần locator còn nằm trực tiếp trong suite</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Locator được chuyển vào Automation/resources/pages/</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Keyword dùng chung</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Nhiều keyword nằm trong test file</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Keyword được tách vào page resource và service resource</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>API/data flow</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Nằm trong remaining_regression.robot</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Đưa vào Automation/resources/services/api_flows.resource</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Kết quả dry-run</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>32/32 Pass</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>32/32 Pass</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>